<commit_message>
Add 11 requested songs to the built-in track list
Imports the September 18 custom-songs export into window.TRACKS so these
play for everyone, not just the device they were added on. Ten go to
Between Whistles and one to Pregame; start times come across unchanged.

Ran through scripts/import_songs_tsv.py, so the block is re-rendered in
the file's own style and round-trip checked before writing. Regenerated
the public track list and the songs spreadsheet from the new block.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164DoZ8Cmq5rP2xy1DrxUaM
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -521,30 +521,34 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Believer</t>
+          <t>Best day of my life</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0pqnGHJpmpxLKifKRmU6WP</t>
+          <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr"/>
+          <t>Pregame</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>2:34</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Ready for It?</t>
+          <t>Believer</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2yLa0QULdQr0qAIvVwN6B5</t>
+          <t>https://open.spotify.com/track/0pqnGHJpmpxLKifKRmU6WP</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -552,21 +556,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>0:08</t>
-        </is>
-      </c>
+      <c r="D5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Let's Go</t>
+          <t>Ready for It?</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6RSuGXM9GVMdXaI8ifGm8d</t>
+          <t>https://open.spotify.com/track/2yLa0QULdQr0qAIvVwN6B5</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -574,17 +574,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>0:08</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Centuries</t>
+          <t>Let's Go</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/04aAxqtGp5pv12UXAg4pkq</t>
+          <t>https://open.spotify.com/track/6RSuGXM9GVMdXaI8ifGm8d</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -592,21 +596,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>0:25</t>
-        </is>
-      </c>
+      <c r="D7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Turn Down for What</t>
+          <t>Centuries</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/67awxiNHNyjMXhVgsHuIrs</t>
+          <t>https://open.spotify.com/track/04aAxqtGp5pv12UXAg4pkq</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -616,19 +616,19 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>0:16</t>
+          <t>0:25</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Danger Zone</t>
+          <t>Turn Down for What</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/34x6hEJgGAOQvmlMql5Ige</t>
+          <t>https://open.spotify.com/track/67awxiNHNyjMXhVgsHuIrs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -638,19 +638,19 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>0:53</t>
+          <t>0:16</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Tick Tick Boom</t>
+          <t>Danger Zone</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5nKdxWYQJTzJrHXWOSO9tO</t>
+          <t>https://open.spotify.com/track/34x6hEJgGAOQvmlMql5Ige</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -660,19 +660,19 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>0:12</t>
+          <t>0:53</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>The Hockey Song</t>
+          <t>Tick Tick Boom</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2g8q4vNuoVpLJGK17kVcoR</t>
+          <t>https://open.spotify.com/track/5nKdxWYQJTzJrHXWOSO9tO</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -680,17 +680,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>0:12</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Unstoppable</t>
+          <t>The Hockey Song</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1yvMUkIOTeUNtNWlWRgANS</t>
+          <t>https://open.spotify.com/track/2g8q4vNuoVpLJGK17kVcoR</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -698,21 +702,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>3:05</t>
-        </is>
-      </c>
+      <c r="D12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Espresso</t>
+          <t>Unstoppable</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1vLqigPHwiFnXsfrLMehV1</t>
+          <t>https://open.spotify.com/track/1yvMUkIOTeUNtNWlWRgANS</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -722,19 +722,19 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>0:08</t>
+          <t>3:05</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Let's Get It Started</t>
+          <t>Espresso</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0EAARxHiL76Us70njzbItJ</t>
+          <t>https://open.spotify.com/track/1vLqigPHwiFnXsfrLMehV1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -744,19 +744,19 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>0:50</t>
+          <t>0:08</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>brutal</t>
+          <t>Let's Get It Started</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6SRsiMl7w1USE4mFqrOhHC</t>
+          <t>https://open.spotify.com/track/0EAARxHiL76Us70njzbItJ</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -766,19 +766,19 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>1:00</t>
+          <t>0:50</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kisses 1</t>
+          <t>brutal</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2A1aS3mwuGuX2yk1bgxOvA</t>
+          <t>https://open.spotify.com/track/6SRsiMl7w1USE4mFqrOhHC</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -788,19 +788,19 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>0:35</t>
+          <t>1:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Wild child</t>
+          <t>Kisses 1</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/02bJ6uGeHKfNOhIc9qyA8e</t>
+          <t>https://open.spotify.com/track/2A1aS3mwuGuX2yk1bgxOvA</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -810,19 +810,19 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2:02</t>
+          <t>0:35</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Runaway</t>
+          <t>Wild child</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4Nh7Umpl8YPFPcggcby6JW</t>
+          <t>https://open.spotify.com/track/02bJ6uGeHKfNOhIc9qyA8e</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -832,19 +832,19 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>0:45</t>
+          <t>2:02</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Chelsea dagger</t>
+          <t>Runaway</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0txisWocI2H8yPRjYxLo83</t>
+          <t>https://open.spotify.com/track/4Nh7Umpl8YPFPcggcby6JW</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>3:06</t>
+          <t>0:45</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Shoot to Thrill</t>
+          <t>Chelsea dagger</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0C80GCp0mMuBzLf3EAXqxv</t>
+          <t>https://open.spotify.com/track/0txisWocI2H8yPRjYxLo83</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -876,19 +876,19 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>1:02</t>
+          <t>3:06</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>9 to 5</t>
+          <t>Shoot to Thrill</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4w3tQBXhn5345eUXDGBWZG</t>
+          <t>https://open.spotify.com/track/0C80GCp0mMuBzLf3EAXqxv</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -898,19 +898,19 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>1:28</t>
+          <t>1:02</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Lush Life</t>
+          <t>9 to 5</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0e6WPtkB9dwFiwspkEeen2</t>
+          <t>https://open.spotify.com/track/4w3tQBXhn5345eUXDGBWZG</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -920,19 +920,19 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>0:49</t>
+          <t>1:28</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>pink pony club</t>
+          <t>Lush Life</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1k2pQc5i348DCHwbn5KTdc</t>
+          <t>https://open.spotify.com/track/0e6WPtkB9dwFiwspkEeen2</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -942,19 +942,19 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2:15</t>
+          <t>0:49</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>the distance</t>
+          <t>pink pony club</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1szwDbVdIdoQq5mG5GXAmJ</t>
+          <t>https://open.spotify.com/track/1k2pQc5i348DCHwbn5KTdc</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -964,19 +964,19 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>0:42</t>
+          <t>2:15</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>wild thing</t>
+          <t>the distance</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/01lZlV0coZWuhzZpFQZ43u</t>
+          <t>https://open.spotify.com/track/1szwDbVdIdoQq5mG5GXAmJ</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -984,17 +984,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>0:42</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>brass</t>
+          <t>wild thing</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/03ZyPqIZXdBNNVIpM2KORq</t>
+          <t>https://open.spotify.com/track/01lZlV0coZWuhzZpFQZ43u</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1002,21 +1006,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
-      </c>
+      <c r="D26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>get ready for this</t>
+          <t>brass</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5zyxpZ8xZmTuhXOuZq4KBG</t>
+          <t>https://open.spotify.com/track/03ZyPqIZXdBNNVIpM2KORq</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1026,19 +1026,19 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>0:25</t>
+          <t>0:30</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>handclap</t>
+          <t>get ready for this</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0y3fi7fknIXOxnkbUgzT3n</t>
+          <t>https://open.spotify.com/track/5zyxpZ8xZmTuhXOuZq4KBG</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1048,19 +1048,19 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>0:27</t>
+          <t>0:25</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>rock n roll gary glitter</t>
+          <t>handclap</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1t3mzpCfaMsEqL1Fbq46ST</t>
+          <t>https://open.spotify.com/track/0y3fi7fknIXOxnkbUgzT3n</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1070,19 +1070,19 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>0:44</t>
+          <t>0:27</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>legend</t>
+          <t>rock n roll gary glitter</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3SWqGa1J0M7hSBUDM0KePD</t>
+          <t>https://open.spotify.com/track/1t3mzpCfaMsEqL1Fbq46ST</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1092,239 +1092,879 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>0:16</t>
+          <t>0:44</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Thunderstruck</t>
+          <t>legend</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
+          <t>https://open.spotify.com/track/3SWqGa1J0M7hSBUDM0KePD</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>2:38</t>
+          <t>0:16</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Kickstart my Heart</t>
+          <t>You Make My Dreams (Come True)</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
+          <t>https://open.spotify.com/track/4o6BgsqLIBViaGVbx5rbRk</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>1:03</t>
-        </is>
-      </c>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Shake it Off</t>
+          <t>Kernkraft 400</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
+          <t>https://open.spotify.com/track/3f2fyR55BFMl3ZWS5S3BUZ</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>0:41</t>
+          <t>1:56</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>We're not gonna take it</t>
+          <t>Song 2</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
+          <t>https://open.spotify.com/track/1FTSo4v6BOZH9QxKc3MbVM</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>0:46</t>
+          <t>0:14</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Fireball</t>
+          <t>Jump Around</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+          <t>https://open.spotify.com/track/6JymsaWDHk2Yj4e0yNBIFH</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Powerplay</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>1:32</t>
-        </is>
-      </c>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>I Did Something Bad</t>
+          <t>Party Till We Die</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
+          <t>https://open.spotify.com/track/5AEs83CYoPApEjYEJGbTuJ</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>0:44</t>
-        </is>
-      </c>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Bad Girls</t>
+          <t>Bye Bye Bye</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
+          <t>https://open.spotify.com/track/4r8lRYnoOGdEi6YyI5OC1o</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>1:33</t>
+          <t>0:54</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Final Countdown</t>
+          <t>Crazy Train</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+          <t>https://open.spotify.com/track/7ACxUo21jtTHzy7ZEV56vU</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>End Game Intensity</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>4:08</t>
-        </is>
-      </c>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Knights of Cydonia</t>
+          <t>Eye of the Tiger</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
+          <t>https://open.spotify.com/track/2HHtWyy5CgaQbC7XSoOb0e</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>End Game Intensity</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>4:10</t>
-        </is>
-      </c>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>I Wanna Dance with Somebody</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/2tUBqZG2AbRi7Q0BIrVrEj</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>1:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>I Am Your Gummy Bear</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/6nFYXpBgrNcZjbtNEuc6yR</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>0:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Narco</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/4TuNI3WEMyLQAKRMJmcQdA</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Thunder</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/1zB4vmk8tFRmM9UULNzbLB</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>1:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Miles On It</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/4pkb8SbRGeHAvdb87v9rpf</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>2:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/05RgAMGypEvqhNs5hPCbMS</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Papi</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/0VoH8AGgoJ20DmTeEEOBAU</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Celebration</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3K7Q9PHUWPTaknlbFPThn2</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Hall of Fame</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/7wMq5n8mYSKlQIGECKUgTX</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Seven Nation Army</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3dPQuX8Gs42Y7b454ybpMR</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Freaks</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/44DCjBHfvn5s6ZfLHpKmBi</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Play Hard</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/5YPMEOJ58kfl56VHxTgwx3</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>The Gambler</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/5KqldkCunQ2rWxruMEtGh0</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Born to be Wild</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/2VPGmrcBw5X4yAu3B8UZNE</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>1:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Wild side</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/7zVpUAOuXY7pHHSm21jFEq</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>2:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Wild one</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/1NpW5kyvO4XrNJ3rnfcNy3</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>2:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Best day of my life</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>2:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Sharp dressed man</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/0bRNszTbTFLNlunAeh7eom</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Hot to Go</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/4xdBrk0nFZaP54vvZj0yx7</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>1:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Giddy up</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/4NdJlsPyvXz15LySCNoL2W</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>0:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Man i feel like a woman</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/6sxptembJVty4sNtcPMAVz</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Venga Bus</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/73ljrkSg4A0q3ByU0Cu7mw</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>1:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Ceiling can't hold us</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/22skzmqfdWrjJylampe0kt</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>3:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Thunderstruck</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Goal FOR</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>2:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Kickstart my Heart</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Goal FOR</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>1:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Shake it Off</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Goal AGAINST</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>0:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>We're not gonna take it</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Goal AGAINST</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>0:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Fireball</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Powerplay</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>1:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>I Did Something Bad</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Penalty Kill</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>0:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Bad Girls</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Penalty Kill</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>1:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Final Countdown</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>End Game Intensity</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>4:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Knights of Cydonia</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>End Game Intensity</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
           <t>Immigrant Song</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>https://open.spotify.com/track/78lgmZwycJ3nzsdgmPPGNx</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>End Game Intensity</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr">
         <is>
           <t>0:01</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.TRACKS block in index.html. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D40"/>
+  <autoFilter ref="A1:D72"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -1365,6 +2005,38 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId71"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Empty the Pregame list so no song is stranded behind that button
The Pregame button plays an uploaded announcement file whenever one is
loaded, and only falls back to the Spotify list when none is, so the
songs listed under Pregame were unreachable on a device with a file
uploaded.

All three were already in Between Whistles under the same Spotify track,
so nothing needed copying across: 'Pregame Track' is the same track as
'Believer' there, 'brutal' was identical, and 'Best day of my life' is
there two seconds earlier at 2:32 rather than 2:34. The three duplicate
entries are dropped rather than moved, which keeps the selector from
listing the same song twice.

Regenerated the public track list and the spreadsheet: 71 -> 68 songs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164DoZ8Cmq5rP2xy1DrxUaM
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pregame Track</t>
+          <t>Believer</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -491,7 +491,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Pregame</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr"/>
@@ -499,56 +499,52 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>brutal</t>
+          <t>Ready for It?</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6SRsiMl7w1USE4mFqrOhHC</t>
+          <t>https://open.spotify.com/track/2yLa0QULdQr0qAIvVwN6B5</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Pregame</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1:00</t>
+          <t>0:08</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Best day of my life</t>
+          <t>Let's Go</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
+          <t>https://open.spotify.com/track/6RSuGXM9GVMdXaI8ifGm8d</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Pregame</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>2:34</t>
-        </is>
-      </c>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Believer</t>
+          <t>Centuries</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0pqnGHJpmpxLKifKRmU6WP</t>
+          <t>https://open.spotify.com/track/04aAxqtGp5pv12UXAg4pkq</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -556,17 +552,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>0:25</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Ready for It?</t>
+          <t>Turn Down for What</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2yLa0QULdQr0qAIvVwN6B5</t>
+          <t>https://open.spotify.com/track/67awxiNHNyjMXhVgsHuIrs</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -576,19 +576,19 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>0:08</t>
+          <t>0:16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Let's Go</t>
+          <t>Danger Zone</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6RSuGXM9GVMdXaI8ifGm8d</t>
+          <t>https://open.spotify.com/track/34x6hEJgGAOQvmlMql5Ige</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -596,17 +596,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>0:53</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Centuries</t>
+          <t>Tick Tick Boom</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/04aAxqtGp5pv12UXAg4pkq</t>
+          <t>https://open.spotify.com/track/5nKdxWYQJTzJrHXWOSO9tO</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -616,19 +620,19 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>0:25</t>
+          <t>0:12</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Turn Down for What</t>
+          <t>The Hockey Song</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/67awxiNHNyjMXhVgsHuIrs</t>
+          <t>https://open.spotify.com/track/2g8q4vNuoVpLJGK17kVcoR</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -636,21 +640,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>0:16</t>
-        </is>
-      </c>
+      <c r="D9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Danger Zone</t>
+          <t>Unstoppable</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/34x6hEJgGAOQvmlMql5Ige</t>
+          <t>https://open.spotify.com/track/1yvMUkIOTeUNtNWlWRgANS</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -660,19 +660,19 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>0:53</t>
+          <t>3:05</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Tick Tick Boom</t>
+          <t>Espresso</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5nKdxWYQJTzJrHXWOSO9tO</t>
+          <t>https://open.spotify.com/track/1vLqigPHwiFnXsfrLMehV1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -682,19 +682,19 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>0:12</t>
+          <t>0:08</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>The Hockey Song</t>
+          <t>Let's Get It Started</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2g8q4vNuoVpLJGK17kVcoR</t>
+          <t>https://open.spotify.com/track/0EAARxHiL76Us70njzbItJ</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -702,17 +702,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>0:50</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Unstoppable</t>
+          <t>brutal</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1yvMUkIOTeUNtNWlWRgANS</t>
+          <t>https://open.spotify.com/track/6SRsiMl7w1USE4mFqrOhHC</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -722,19 +726,19 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>3:05</t>
+          <t>1:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Espresso</t>
+          <t>Kisses 1</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1vLqigPHwiFnXsfrLMehV1</t>
+          <t>https://open.spotify.com/track/2A1aS3mwuGuX2yk1bgxOvA</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -744,19 +748,19 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>0:08</t>
+          <t>0:35</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Let's Get It Started</t>
+          <t>Wild child</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0EAARxHiL76Us70njzbItJ</t>
+          <t>https://open.spotify.com/track/02bJ6uGeHKfNOhIc9qyA8e</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -766,19 +770,19 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>0:50</t>
+          <t>2:02</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>brutal</t>
+          <t>Runaway</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6SRsiMl7w1USE4mFqrOhHC</t>
+          <t>https://open.spotify.com/track/4Nh7Umpl8YPFPcggcby6JW</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -788,19 +792,19 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>1:00</t>
+          <t>0:45</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kisses 1</t>
+          <t>Chelsea dagger</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2A1aS3mwuGuX2yk1bgxOvA</t>
+          <t>https://open.spotify.com/track/0txisWocI2H8yPRjYxLo83</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -810,19 +814,19 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>0:35</t>
+          <t>3:06</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Wild child</t>
+          <t>Shoot to Thrill</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/02bJ6uGeHKfNOhIc9qyA8e</t>
+          <t>https://open.spotify.com/track/0C80GCp0mMuBzLf3EAXqxv</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -832,19 +836,19 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2:02</t>
+          <t>1:02</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Runaway</t>
+          <t>9 to 5</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4Nh7Umpl8YPFPcggcby6JW</t>
+          <t>https://open.spotify.com/track/4w3tQBXhn5345eUXDGBWZG</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -854,19 +858,19 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>0:45</t>
+          <t>1:28</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Chelsea dagger</t>
+          <t>Lush Life</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0txisWocI2H8yPRjYxLo83</t>
+          <t>https://open.spotify.com/track/0e6WPtkB9dwFiwspkEeen2</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -876,19 +880,19 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>3:06</t>
+          <t>0:49</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Shoot to Thrill</t>
+          <t>pink pony club</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0C80GCp0mMuBzLf3EAXqxv</t>
+          <t>https://open.spotify.com/track/1k2pQc5i348DCHwbn5KTdc</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -898,19 +902,19 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>1:02</t>
+          <t>2:15</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>9 to 5</t>
+          <t>the distance</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4w3tQBXhn5345eUXDGBWZG</t>
+          <t>https://open.spotify.com/track/1szwDbVdIdoQq5mG5GXAmJ</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -920,19 +924,19 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>1:28</t>
+          <t>0:42</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Lush Life</t>
+          <t>wild thing</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0e6WPtkB9dwFiwspkEeen2</t>
+          <t>https://open.spotify.com/track/01lZlV0coZWuhzZpFQZ43u</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -940,21 +944,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>0:49</t>
-        </is>
-      </c>
+      <c r="D23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>pink pony club</t>
+          <t>brass</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1k2pQc5i348DCHwbn5KTdc</t>
+          <t>https://open.spotify.com/track/03ZyPqIZXdBNNVIpM2KORq</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -964,19 +964,19 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2:15</t>
+          <t>0:30</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>the distance</t>
+          <t>get ready for this</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1szwDbVdIdoQq5mG5GXAmJ</t>
+          <t>https://open.spotify.com/track/5zyxpZ8xZmTuhXOuZq4KBG</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -986,19 +986,19 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>0:42</t>
+          <t>0:25</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>wild thing</t>
+          <t>handclap</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/01lZlV0coZWuhzZpFQZ43u</t>
+          <t>https://open.spotify.com/track/0y3fi7fknIXOxnkbUgzT3n</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1006,17 +1006,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>0:27</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>brass</t>
+          <t>rock n roll gary glitter</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/03ZyPqIZXdBNNVIpM2KORq</t>
+          <t>https://open.spotify.com/track/1t3mzpCfaMsEqL1Fbq46ST</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1026,19 +1030,19 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>0:30</t>
+          <t>0:44</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>get ready for this</t>
+          <t>legend</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5zyxpZ8xZmTuhXOuZq4KBG</t>
+          <t>https://open.spotify.com/track/3SWqGa1J0M7hSBUDM0KePD</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1048,19 +1052,19 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>0:25</t>
+          <t>0:16</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>handclap</t>
+          <t>You Make My Dreams (Come True)</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0y3fi7fknIXOxnkbUgzT3n</t>
+          <t>https://open.spotify.com/track/4o6BgsqLIBViaGVbx5rbRk</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1068,21 +1072,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>0:27</t>
-        </is>
-      </c>
+      <c r="D29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>rock n roll gary glitter</t>
+          <t>Kernkraft 400</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1t3mzpCfaMsEqL1Fbq46ST</t>
+          <t>https://open.spotify.com/track/3f2fyR55BFMl3ZWS5S3BUZ</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1092,19 +1092,19 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>0:44</t>
+          <t>1:56</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>legend</t>
+          <t>Song 2</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3SWqGa1J0M7hSBUDM0KePD</t>
+          <t>https://open.spotify.com/track/1FTSo4v6BOZH9QxKc3MbVM</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1114,19 +1114,19 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>0:16</t>
+          <t>0:14</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>You Make My Dreams (Come True)</t>
+          <t>Jump Around</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4o6BgsqLIBViaGVbx5rbRk</t>
+          <t>https://open.spotify.com/track/6JymsaWDHk2Yj4e0yNBIFH</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1139,12 +1139,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Kernkraft 400</t>
+          <t>Party Till We Die</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3f2fyR55BFMl3ZWS5S3BUZ</t>
+          <t>https://open.spotify.com/track/5AEs83CYoPApEjYEJGbTuJ</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1152,21 +1152,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>1:56</t>
-        </is>
-      </c>
+      <c r="D33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Song 2</t>
+          <t>Bye Bye Bye</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1FTSo4v6BOZH9QxKc3MbVM</t>
+          <t>https://open.spotify.com/track/4r8lRYnoOGdEi6YyI5OC1o</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1176,19 +1172,19 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>0:14</t>
+          <t>0:54</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Jump Around</t>
+          <t>Crazy Train</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6JymsaWDHk2Yj4e0yNBIFH</t>
+          <t>https://open.spotify.com/track/7ACxUo21jtTHzy7ZEV56vU</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1201,12 +1197,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Party Till We Die</t>
+          <t>Eye of the Tiger</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5AEs83CYoPApEjYEJGbTuJ</t>
+          <t>https://open.spotify.com/track/2HHtWyy5CgaQbC7XSoOb0e</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1219,12 +1215,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Bye Bye Bye</t>
+          <t>I Wanna Dance with Somebody</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4r8lRYnoOGdEi6YyI5OC1o</t>
+          <t>https://open.spotify.com/track/2tUBqZG2AbRi7Q0BIrVrEj</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1234,19 +1230,19 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>0:54</t>
+          <t>1:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Crazy Train</t>
+          <t>I Am Your Gummy Bear</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7ACxUo21jtTHzy7ZEV56vU</t>
+          <t>https://open.spotify.com/track/6nFYXpBgrNcZjbtNEuc6yR</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1254,17 +1250,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>0:37</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Eye of the Tiger</t>
+          <t>Narco</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2HHtWyy5CgaQbC7XSoOb0e</t>
+          <t>https://open.spotify.com/track/4TuNI3WEMyLQAKRMJmcQdA</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1277,12 +1277,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>I Wanna Dance with Somebody</t>
+          <t>Thunder</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2tUBqZG2AbRi7Q0BIrVrEj</t>
+          <t>https://open.spotify.com/track/1zB4vmk8tFRmM9UULNzbLB</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1292,19 +1292,19 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>1:00</t>
+          <t>1:13</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>I Am Your Gummy Bear</t>
+          <t>Miles On It</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6nFYXpBgrNcZjbtNEuc6yR</t>
+          <t>https://open.spotify.com/track/4pkb8SbRGeHAvdb87v9rpf</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -1314,19 +1314,19 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>0:37</t>
+          <t>2:12</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Narco</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4TuNI3WEMyLQAKRMJmcQdA</t>
+          <t>https://open.spotify.com/track/05RgAMGypEvqhNs5hPCbMS</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -1339,12 +1339,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Thunder</t>
+          <t>Papi</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1zB4vmk8tFRmM9UULNzbLB</t>
+          <t>https://open.spotify.com/track/0VoH8AGgoJ20DmTeEEOBAU</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1352,21 +1352,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>1:13</t>
-        </is>
-      </c>
+      <c r="D43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Miles On It</t>
+          <t>Celebration</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4pkb8SbRGeHAvdb87v9rpf</t>
+          <t>https://open.spotify.com/track/3K7Q9PHUWPTaknlbFPThn2</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -1374,21 +1370,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>2:12</t>
-        </is>
-      </c>
+      <c r="D44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Hall of Fame</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/05RgAMGypEvqhNs5hPCbMS</t>
+          <t>https://open.spotify.com/track/7wMq5n8mYSKlQIGECKUgTX</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -1401,12 +1393,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Papi</t>
+          <t>Seven Nation Army</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0VoH8AGgoJ20DmTeEEOBAU</t>
+          <t>https://open.spotify.com/track/3dPQuX8Gs42Y7b454ybpMR</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -1419,12 +1411,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Celebration</t>
+          <t>Freaks</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3K7Q9PHUWPTaknlbFPThn2</t>
+          <t>https://open.spotify.com/track/44DCjBHfvn5s6ZfLHpKmBi</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -1437,12 +1429,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Hall of Fame</t>
+          <t>Play Hard</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7wMq5n8mYSKlQIGECKUgTX</t>
+          <t>https://open.spotify.com/track/5YPMEOJ58kfl56VHxTgwx3</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -1455,12 +1447,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Seven Nation Army</t>
+          <t>The Gambler</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3dPQuX8Gs42Y7b454ybpMR</t>
+          <t>https://open.spotify.com/track/5KqldkCunQ2rWxruMEtGh0</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -1473,12 +1465,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Freaks</t>
+          <t>Born to be Wild</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/44DCjBHfvn5s6ZfLHpKmBi</t>
+          <t>https://open.spotify.com/track/2VPGmrcBw5X4yAu3B8UZNE</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -1486,17 +1478,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>1:08</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Play Hard</t>
+          <t>Wild side</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5YPMEOJ58kfl56VHxTgwx3</t>
+          <t>https://open.spotify.com/track/7zVpUAOuXY7pHHSm21jFEq</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -1504,17 +1500,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>2:46</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>The Gambler</t>
+          <t>Wild one</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5KqldkCunQ2rWxruMEtGh0</t>
+          <t>https://open.spotify.com/track/1NpW5kyvO4XrNJ3rnfcNy3</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -1522,17 +1522,21 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr"/>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>2:02</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Born to be Wild</t>
+          <t>Best day of my life</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2VPGmrcBw5X4yAu3B8UZNE</t>
+          <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -1542,19 +1546,19 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>1:08</t>
+          <t>2:32</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Wild side</t>
+          <t>Sharp dressed man</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7zVpUAOuXY7pHHSm21jFEq</t>
+          <t>https://open.spotify.com/track/0bRNszTbTFLNlunAeh7eom</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -1562,21 +1566,17 @@
           <t>Between Whistles</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>2:46</t>
-        </is>
-      </c>
+      <c r="D54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Wild one</t>
+          <t>Hot to Go</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1NpW5kyvO4XrNJ3rnfcNy3</t>
+          <t>https://open.spotify.com/track/4xdBrk0nFZaP54vvZj0yx7</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -1586,19 +1586,19 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>2:02</t>
+          <t>1:53</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Best day of my life</t>
+          <t>Giddy up</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
+          <t>https://open.spotify.com/track/4NdJlsPyvXz15LySCNoL2W</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -1608,19 +1608,19 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>2:32</t>
+          <t>0:32</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Sharp dressed man</t>
+          <t>Man i feel like a woman</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0bRNszTbTFLNlunAeh7eom</t>
+          <t>https://open.spotify.com/track/6sxptembJVty4sNtcPMAVz</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -1633,12 +1633,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Hot to Go</t>
+          <t>Venga Bus</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4xdBrk0nFZaP54vvZj0yx7</t>
+          <t>https://open.spotify.com/track/73ljrkSg4A0q3ByU0Cu7mw</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -1648,19 +1648,19 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>1:53</t>
+          <t>1:09</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Giddy up</t>
+          <t>Ceiling can't hold us</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4NdJlsPyvXz15LySCNoL2W</t>
+          <t>https://open.spotify.com/track/22skzmqfdWrjJylampe0kt</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -1670,301 +1670,239 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>0:32</t>
+          <t>3:49</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Man i feel like a woman</t>
+          <t>Thunderstruck</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6sxptembJVty4sNtcPMAVz</t>
+          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="inlineStr"/>
+          <t>Goal FOR</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>2:38</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Venga Bus</t>
+          <t>Kickstart my Heart</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/73ljrkSg4A0q3ByU0Cu7mw</t>
+          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Between Whistles</t>
+          <t>Goal FOR</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1:09</t>
+          <t>1:03</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Ceiling can't hold us</t>
+          <t>Shake it Off</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/22skzmqfdWrjJylampe0kt</t>
+          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Between Whistles</t>
+          <t>Goal AGAINST</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>3:49</t>
+          <t>0:41</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Thunderstruck</t>
+          <t>We're not gonna take it</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
+          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
+          <t>Goal AGAINST</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>2:38</t>
+          <t>0:46</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Kickstart my Heart</t>
+          <t>Fireball</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
+          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
+          <t>Powerplay</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>1:03</t>
+          <t>1:32</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Shake it Off</t>
+          <t>I Did Something Bad</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
+          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Penalty Kill</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>0:41</t>
+          <t>0:44</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>We're not gonna take it</t>
+          <t>Bad Girls</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
+          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Penalty Kill</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>0:46</t>
+          <t>1:33</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Fireball</t>
+          <t>Final Countdown</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Powerplay</t>
+          <t>End Game Intensity</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>1:32</t>
+          <t>4:08</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>I Did Something Bad</t>
+          <t>Knights of Cydonia</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
+          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
+          <t>End Game Intensity</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>0:44</t>
+          <t>4:10</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Bad Girls</t>
+          <t>Immigrant Song</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
+          <t>https://open.spotify.com/track/78lgmZwycJ3nzsdgmPPGNx</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
+          <t>End Game Intensity</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>1:33</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Final Countdown</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>End Game Intensity</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>4:08</t>
+          <t>0:01</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>Knights of Cydonia</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>End Game Intensity</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>4:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>Immigrant Song</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>https://open.spotify.com/track/78lgmZwycJ3nzsdgmPPGNx</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>End Game Intensity</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>0:01</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="5" t="inlineStr">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.TRACKS block in index.html. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D72"/>
+  <autoFilter ref="A1:D69"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2034,9 +1972,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId71"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Flat song list: one list with optional tags, no Between Whistles category
Songs carry tags (Power Play, Goal For, Goal Against, Penalty Kill, End Game);
untagged songs are between-whistles songs. Add Custom Song form now has link,
name, start time and multi-select tag chips. Old on-device data and export
files convert automatically. Scripts, track list page and spreadsheet updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Tags</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -489,11 +489,7 @@
           <t>https://open.spotify.com/track/0pqnGHJpmpxLKifKRmU6WP</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
@@ -507,11 +503,7 @@
           <t>https://open.spotify.com/track/2yLa0QULdQr0qAIvVwN6B5</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>0:08</t>
@@ -529,11 +521,7 @@
           <t>https://open.spotify.com/track/6RSuGXM9GVMdXaI8ifGm8d</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -547,11 +535,7 @@
           <t>https://open.spotify.com/track/04aAxqtGp5pv12UXAg4pkq</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>0:25</t>
@@ -569,11 +553,7 @@
           <t>https://open.spotify.com/track/67awxiNHNyjMXhVgsHuIrs</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
           <t>0:16</t>
@@ -591,11 +571,7 @@
           <t>https://open.spotify.com/track/34x6hEJgGAOQvmlMql5Ige</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
           <t>0:53</t>
@@ -613,11 +589,7 @@
           <t>https://open.spotify.com/track/5nKdxWYQJTzJrHXWOSO9tO</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
           <t>0:12</t>
@@ -635,11 +607,7 @@
           <t>https://open.spotify.com/track/2g8q4vNuoVpLJGK17kVcoR</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
@@ -653,11 +621,7 @@
           <t>https://open.spotify.com/track/1yvMUkIOTeUNtNWlWRgANS</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="4" t="inlineStr">
         <is>
           <t>3:05</t>
@@ -675,11 +639,7 @@
           <t>https://open.spotify.com/track/1vLqigPHwiFnXsfrLMehV1</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
           <t>0:08</t>
@@ -697,11 +657,7 @@
           <t>https://open.spotify.com/track/0EAARxHiL76Us70njzbItJ</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="4" t="inlineStr">
         <is>
           <t>0:50</t>
@@ -719,11 +675,7 @@
           <t>https://open.spotify.com/track/6SRsiMl7w1USE4mFqrOhHC</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr">
         <is>
           <t>1:00</t>
@@ -741,11 +693,7 @@
           <t>https://open.spotify.com/track/2A1aS3mwuGuX2yk1bgxOvA</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
           <t>0:35</t>
@@ -763,11 +711,7 @@
           <t>https://open.spotify.com/track/02bJ6uGeHKfNOhIc9qyA8e</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr">
         <is>
           <t>2:02</t>
@@ -785,11 +729,7 @@
           <t>https://open.spotify.com/track/4Nh7Umpl8YPFPcggcby6JW</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="4" t="inlineStr">
         <is>
           <t>0:45</t>
@@ -807,11 +747,7 @@
           <t>https://open.spotify.com/track/0txisWocI2H8yPRjYxLo83</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr">
         <is>
           <t>3:06</t>
@@ -829,11 +765,7 @@
           <t>https://open.spotify.com/track/0C80GCp0mMuBzLf3EAXqxv</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="4" t="inlineStr">
         <is>
           <t>1:02</t>
@@ -851,11 +783,7 @@
           <t>https://open.spotify.com/track/4w3tQBXhn5345eUXDGBWZG</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr">
         <is>
           <t>1:28</t>
@@ -873,11 +801,7 @@
           <t>https://open.spotify.com/track/0e6WPtkB9dwFiwspkEeen2</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="4" t="inlineStr">
         <is>
           <t>0:49</t>
@@ -895,11 +819,7 @@
           <t>https://open.spotify.com/track/1k2pQc5i348DCHwbn5KTdc</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="4" t="inlineStr">
         <is>
           <t>2:15</t>
@@ -917,11 +837,7 @@
           <t>https://open.spotify.com/track/1szwDbVdIdoQq5mG5GXAmJ</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="4" t="inlineStr">
         <is>
           <t>0:42</t>
@@ -939,11 +855,7 @@
           <t>https://open.spotify.com/track/01lZlV0coZWuhzZpFQZ43u</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
@@ -957,11 +869,7 @@
           <t>https://open.spotify.com/track/03ZyPqIZXdBNNVIpM2KORq</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="4" t="inlineStr">
         <is>
           <t>0:30</t>
@@ -979,11 +887,7 @@
           <t>https://open.spotify.com/track/5zyxpZ8xZmTuhXOuZq4KBG</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="4" t="inlineStr">
         <is>
           <t>0:25</t>
@@ -1001,11 +905,7 @@
           <t>https://open.spotify.com/track/0y3fi7fknIXOxnkbUgzT3n</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="4" t="inlineStr">
         <is>
           <t>0:27</t>
@@ -1023,11 +923,7 @@
           <t>https://open.spotify.com/track/1t3mzpCfaMsEqL1Fbq46ST</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="4" t="inlineStr">
         <is>
           <t>0:44</t>
@@ -1045,11 +941,7 @@
           <t>https://open.spotify.com/track/3SWqGa1J0M7hSBUDM0KePD</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="4" t="inlineStr">
         <is>
           <t>0:16</t>
@@ -1067,11 +959,7 @@
           <t>https://open.spotify.com/track/4o6BgsqLIBViaGVbx5rbRk</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1085,11 +973,7 @@
           <t>https://open.spotify.com/track/3f2fyR55BFMl3ZWS5S3BUZ</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="4" t="inlineStr">
         <is>
           <t>1:56</t>
@@ -1107,11 +991,7 @@
           <t>https://open.spotify.com/track/1FTSo4v6BOZH9QxKc3MbVM</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="4" t="inlineStr">
         <is>
           <t>0:14</t>
@@ -1129,11 +1009,7 @@
           <t>https://open.spotify.com/track/6JymsaWDHk2Yj4e0yNBIFH</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1147,11 +1023,7 @@
           <t>https://open.spotify.com/track/5AEs83CYoPApEjYEJGbTuJ</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C33" s="2" t="inlineStr"/>
       <c r="D33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1165,11 +1037,7 @@
           <t>https://open.spotify.com/track/4r8lRYnoOGdEi6YyI5OC1o</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="4" t="inlineStr">
         <is>
           <t>0:54</t>
@@ -1187,11 +1055,7 @@
           <t>https://open.spotify.com/track/7ACxUo21jtTHzy7ZEV56vU</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1205,11 +1069,7 @@
           <t>https://open.spotify.com/track/2HHtWyy5CgaQbC7XSoOb0e</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1223,11 +1083,7 @@
           <t>https://open.spotify.com/track/2tUBqZG2AbRi7Q0BIrVrEj</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C37" s="2" t="inlineStr"/>
       <c r="D37" s="4" t="inlineStr">
         <is>
           <t>1:00</t>
@@ -1245,11 +1101,7 @@
           <t>https://open.spotify.com/track/6nFYXpBgrNcZjbtNEuc6yR</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="4" t="inlineStr">
         <is>
           <t>0:37</t>
@@ -1267,11 +1119,7 @@
           <t>https://open.spotify.com/track/4TuNI3WEMyLQAKRMJmcQdA</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1285,11 +1133,7 @@
           <t>https://open.spotify.com/track/1zB4vmk8tFRmM9UULNzbLB</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="4" t="inlineStr">
         <is>
           <t>1:13</t>
@@ -1307,11 +1151,7 @@
           <t>https://open.spotify.com/track/4pkb8SbRGeHAvdb87v9rpf</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="4" t="inlineStr">
         <is>
           <t>2:12</t>
@@ -1329,11 +1169,7 @@
           <t>https://open.spotify.com/track/05RgAMGypEvqhNs5hPCbMS</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C42" s="2" t="inlineStr"/>
       <c r="D42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1347,11 +1183,7 @@
           <t>https://open.spotify.com/track/0VoH8AGgoJ20DmTeEEOBAU</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
@@ -1365,11 +1197,7 @@
           <t>https://open.spotify.com/track/3K7Q9PHUWPTaknlbFPThn2</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
@@ -1383,11 +1211,7 @@
           <t>https://open.spotify.com/track/7wMq5n8mYSKlQIGECKUgTX</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
@@ -1401,11 +1225,7 @@
           <t>https://open.spotify.com/track/3dPQuX8Gs42Y7b454ybpMR</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
@@ -1419,11 +1239,7 @@
           <t>https://open.spotify.com/track/44DCjBHfvn5s6ZfLHpKmBi</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
@@ -1437,11 +1253,7 @@
           <t>https://open.spotify.com/track/5YPMEOJ58kfl56VHxTgwx3</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
@@ -1455,11 +1267,7 @@
           <t>https://open.spotify.com/track/5KqldkCunQ2rWxruMEtGh0</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C49" s="2" t="inlineStr"/>
       <c r="D49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
@@ -1473,11 +1281,7 @@
           <t>https://open.spotify.com/track/2VPGmrcBw5X4yAu3B8UZNE</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="4" t="inlineStr">
         <is>
           <t>1:08</t>
@@ -1495,11 +1299,7 @@
           <t>https://open.spotify.com/track/7zVpUAOuXY7pHHSm21jFEq</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="4" t="inlineStr">
         <is>
           <t>2:46</t>
@@ -1517,11 +1317,7 @@
           <t>https://open.spotify.com/track/1NpW5kyvO4XrNJ3rnfcNy3</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="4" t="inlineStr">
         <is>
           <t>2:02</t>
@@ -1539,11 +1335,7 @@
           <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="4" t="inlineStr">
         <is>
           <t>2:32</t>
@@ -1561,11 +1353,7 @@
           <t>https://open.spotify.com/track/0bRNszTbTFLNlunAeh7eom</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
@@ -1579,11 +1367,7 @@
           <t>https://open.spotify.com/track/4xdBrk0nFZaP54vvZj0yx7</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="4" t="inlineStr">
         <is>
           <t>1:53</t>
@@ -1601,11 +1385,7 @@
           <t>https://open.spotify.com/track/4NdJlsPyvXz15LySCNoL2W</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C56" s="2" t="inlineStr"/>
       <c r="D56" s="4" t="inlineStr">
         <is>
           <t>0:32</t>
@@ -1623,11 +1403,7 @@
           <t>https://open.spotify.com/track/6sxptembJVty4sNtcPMAVz</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C57" s="2" t="inlineStr"/>
       <c r="D57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
@@ -1641,11 +1417,7 @@
           <t>https://open.spotify.com/track/73ljrkSg4A0q3ByU0Cu7mw</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="4" t="inlineStr">
         <is>
           <t>1:09</t>
@@ -1663,11 +1435,7 @@
           <t>https://open.spotify.com/track/22skzmqfdWrjJylampe0kt</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Between Whistles</t>
-        </is>
-      </c>
+      <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="4" t="inlineStr">
         <is>
           <t>3:49</t>
@@ -1687,7 +1455,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
+          <t>Goal For</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -1709,7 +1477,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
+          <t>Goal For</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -1731,7 +1499,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Goal Against</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -1753,7 +1521,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Goal Against</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -1775,7 +1543,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Powerplay</t>
+          <t>Power Play</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -1841,7 +1609,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>End Game Intensity</t>
+          <t>End Game</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -1863,7 +1631,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>End Game Intensity</t>
+          <t>End Game</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -1885,7 +1653,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>End Game Intensity</t>
+          <t>End Game</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -1897,7 +1665,7 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>Exported from the window.TRACKS block in index.html. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
+          <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tag Thunderstruck and Seven Nation Army as Power Play
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -1225,7 +1225,11 @@
           <t>https://open.spotify.com/track/3dPQuX8Gs42Y7b454ybpMR</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Power Play</t>
+        </is>
+      </c>
       <c r="D46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
@@ -1455,7 +1459,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Goal For</t>
+          <t>Power Play, Goal For</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Merge main (Misty Mountain Hop); refresh spreadsheet to 88 songs
AGENTS.md: song-update agents leave wild-hockey-songs.xlsx to Claude.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D90"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2000,15 +2000,29 @@
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="5" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Misty Mountain Hop</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3frf3zTgzt3YIx9ylpUoqU</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr"/>
+      <c r="D89" s="4" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D88"/>
+  <autoFilter ref="A1:D89"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2097,6 +2111,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Song picker: clear (X) button on the right, chips no longer shift
The X now lives outside the scrolling chip area, to the right, and keeps its
space while hidden, so selecting the first chip doesn't move anything.
Also rebuild the track list and spreadsheet for No Broke Boys (89 songs).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2014,15 +2014,33 @@
       <c r="C89" s="2" t="inlineStr"/>
       <c r="D89" s="4" t="inlineStr"/>
     </row>
-    <row r="91">
-      <c r="A91" s="5" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>No Broke Boys</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3cZajhyr8LmtPfHZ9296tj</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr"/>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>0:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D89"/>
+  <autoFilter ref="A1:D90"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2112,6 +2130,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" r:id="rId89"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 4 songs: Goal horn, crowd chant, 50 mission Cap, you've got another thing coming
Goal horn tagged Goal For; crowd chant starts at 0:24. Track list page and
spreadsheet rebuilt (93 songs).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2032,15 +2032,79 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Goal horn</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/7gfcVjQLq4lKObJD6dU7r7</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr"/>
+    </row>
     <row r="92">
-      <c r="A92" s="5" t="inlineStr">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>crowd chant</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/0bz67HYKfiuUj1xhsK5ofT</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr"/>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>0:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>50 mission Cap</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/6UA5wCnNHbPZzT1O0tWQy0</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr"/>
+      <c r="D93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>you've got another thing coming</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/4f3RDq9nYPBeR1yMSgnmBm</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr"/>
+      <c r="D94" s="4" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D90"/>
+  <autoFilter ref="A1:D94"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2131,6 +2195,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" r:id="rId93"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tag 7 songs Goal For: Chelsea dagger, crowd chant, Giddy up, Hot to Go, Panama, Shoot to Thrill, Song 2
Goal For now has 8 songs (with Goal horn). Track list and spreadsheet rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -759,7 +759,11 @@
           <t>https://open.spotify.com/track/0txisWocI2H8yPRjYxLo83</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
           <t>3:06</t>
@@ -777,7 +781,11 @@
           <t>https://open.spotify.com/track/0C80GCp0mMuBzLf3EAXqxv</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
           <t>1:02</t>
@@ -1007,7 +1015,11 @@
           <t>https://open.spotify.com/track/1FTSo4v6BOZH9QxKc3MbVM</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
           <t>0:14</t>
@@ -1193,7 +1205,11 @@
           <t>https://open.spotify.com/track/05RgAMGypEvqhNs5hPCbMS</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
       <c r="D42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1403,7 +1419,11 @@
           <t>https://open.spotify.com/track/4xdBrk0nFZaP54vvZj0yx7</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr"/>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
           <t>1:53</t>
@@ -1421,7 +1441,11 @@
           <t>https://open.spotify.com/track/4NdJlsPyvXz15LySCNoL2W</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr"/>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
           <t>0:32</t>
@@ -2061,7 +2085,11 @@
           <t>https://open.spotify.com/track/0bz67HYKfiuUj1xhsK5ofT</t>
         </is>
       </c>
-      <c r="C92" s="2" t="inlineStr"/>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
           <t>0:24</t>

</xml_diff>

<commit_message>
Tag 5 songs Power Play; add Intensity tag (hot pink, black text)
Power Play: 50 mission Cap, Crazy Train, crowd chant, Fireball, Seek & Destroy
(existing End Game / Goal For tags kept).
Intensity: colour in the app (solid hot pink pill, black text), track list
section, scripts, AGENTS.md and submissions doc. No songs tagged yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -1085,7 +1085,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>End Game</t>
+          <t>Power Play, End Game</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr"/>
@@ -1585,7 +1585,11 @@
           <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr"/>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Power Play</t>
+        </is>
+      </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
           <t>1:32</t>
@@ -1937,7 +1941,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>End Game</t>
+          <t>Power Play, End Game</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr"/>
@@ -2087,7 +2091,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Goal For</t>
+          <t>Power Play, Goal For</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -2107,7 +2111,11 @@
           <t>https://open.spotify.com/track/6UA5wCnNHbPZzT1O0tWQy0</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr"/>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Power Play</t>
+        </is>
+      </c>
       <c r="D93" s="4" t="inlineStr"/>
     </row>
     <row r="94">

</xml_diff>

<commit_message>
Tag 4 songs Penalty Kill; short codes on song-row tag pills
Penalty Kill: Bad Girls, I Did Something Bad, Narco, The Gambler.
Song-row pills now show fixed-width short codes (GF, GA, PP, PK, EG, PD, WLD,
INT) with the full name as a tooltip; filter chips and the data keep full
names. Custom tags without a code show their full name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -1155,7 +1155,11 @@
           <t>https://open.spotify.com/track/4TuNI3WEMyLQAKRMJmcQdA</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Penalty Kill</t>
+        </is>
+      </c>
       <c r="D39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1307,7 +1311,11 @@
           <t>https://open.spotify.com/track/5KqldkCunQ2rWxruMEtGh0</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr"/>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Penalty Kill</t>
+        </is>
+      </c>
       <c r="D49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
@@ -1607,7 +1615,11 @@
           <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr"/>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Penalty Kill</t>
+        </is>
+      </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
           <t>0:44</t>
@@ -1625,7 +1637,11 @@
           <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr"/>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Penalty Kill</t>
+        </is>
+      </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
           <t>1:33</t>

</xml_diff>

<commit_message>
Adjust start times: 9 to 5, Bad Girls, brass, Best day of my life
9 to 5 88 -> 89s; Bad Girls 93 -> 96s; brass 30 -> 32s (+2);
Best day of my life 152 -> 152.5s (+0.5).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -806,7 +806,7 @@
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>1:28</t>
+          <t>1:29</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>0:30</t>
+          <t>0:32</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1398,7 @@
       <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>2:32</t>
+          <t>2:32.5</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>1:33</t>
+          <t>1:36</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
+          <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss (or m:ss.s) and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nudge start times on 9 songs
Billie Jean +1, Born to be Wild +1, brass +1, brutal +0.5, Bye Bye Bye +0.3,
Ceiling can't hold us +0.5, Chelsea dagger +0.5, Danger Zone +1,
Edge of Seventeen +0.5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>0:53</t>
+          <t>0:54</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>1:00</t>
+          <t>1:00.5</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>3:06</t>
+          <t>3:06.5</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>0:32</t>
+          <t>0:33</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>0:54</t>
+          <t>0:54.3</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>1:08</t>
+          <t>1:09</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
       <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>3:49</t>
+          <t>3:49.5</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>4:17</t>
+          <t>4:17.5</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>1:25</t>
+          <t>1:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust start times on 28 songs
Set: Fabienk 4:22, Knights of Cydonia 4:13.2.
Nudged: handclap +2, Final Countdown +3, Hot to Go +0.1, Hangar 18 +0.4,
I Wanna Dance with Somebody +0.4, Kickstart my Heart +0.2, Let's Get It
Started +0.4, Kisses 1 +1.1, Ready for It? +0.8, pink pony club +0.5, Miles
On It +0.3, September +0.2, rock n roll gary glitter +0.3, Shake it Off +0.2,
the distance +0.4, Thunder +0.4, Tick Tick Boom +0.5, Thunderstruck +0.4,
Turn Down for What +0.7, Unstoppable +0.4, Vogue +0.1, Wild child -0.2,
Wild one +0.5, We're not gonna take it +0.5, Wild side +0.1, YYZ +0.2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -506,7 +506,7 @@
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>0:08</t>
+          <t>0:08.8</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>0:16</t>
+          <t>0:16.7</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>0:12</t>
+          <t>0:12.5</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>3:05</t>
+          <t>3:05.4</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>0:50</t>
+          <t>0:50.4</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>0:35</t>
+          <t>0:36.1</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2:02</t>
+          <t>2:01.8</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>2:15</t>
+          <t>2:15.5</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>0:42</t>
+          <t>0:42.4</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>0:27</t>
+          <t>0:29</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>0:44</t>
+          <t>0:44.3</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       <c r="C37" s="2" t="inlineStr"/>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>1:00</t>
+          <t>1:00.4</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>1:13</t>
+          <t>1:13.4</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2:12</t>
+          <t>2:12.3</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>2:46</t>
+          <t>2:46.1</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>2:02</t>
+          <t>2:02.5</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>1:53</t>
+          <t>1:53.1</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>2:38</t>
+          <t>2:38.4</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1:03</t>
+          <t>1:03.2</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>0:41</t>
+          <t>0:41.2</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>0:46</t>
+          <t>0:46.5</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1662,7 @@
       <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>4:08</t>
+          <t>4:11</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1680,7 @@
       <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>4:10</t>
+          <t>4:13.2</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
       <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>4:08</t>
+          <t>4:22</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1734,7 @@
       <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>2:10</t>
+          <t>2:10.2</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>2:43</t>
+          <t>2:43.1</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>0:50</t>
+          <t>0:50.2</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>0:46</t>
+          <t>0:46.4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fine-tune start times on 19 songs
Born to be Wild +0.2, Bye Bye Bye +0.1, Chelsea dagger +0.1, Final Countdown
+0.2, Hangar 18 +0.1, Kickstart my Heart +0.1, Let's Get It Started +0.2,
pink pony club +0.1, rock n roll gary glitter +0.2, Song 2 +0.1, Shoot to
Thrill +0.2, September +0.1, the distance +0.8, Thunder +0.4, Tick Tick Boom
+0.2, Turn Down for What +0.3, Vogue +0.1, We're not gonna take it +0.3,
Wild child -0.1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -556,7 +556,7 @@
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>0:16.7</t>
+          <t>0:17</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>0:12.5</t>
+          <t>0:12.7</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>0:50.4</t>
+          <t>0:50.6</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2:01.8</t>
+          <t>2:01.7</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>3:06.5</t>
+          <t>3:06.6</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>1:02</t>
+          <t>1:02.2</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>2:15.5</t>
+          <t>2:15.6</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>0:42.4</t>
+          <t>0:43.2</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>0:44.3</t>
+          <t>0:44.5</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>0:14</t>
+          <t>0:14.1</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>0:54.3</t>
+          <t>0:54.4</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>1:13.4</t>
+          <t>1:13.8</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>1:09</t>
+          <t>1:09.2</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1:03.2</t>
+          <t>1:03.3</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>0:46.5</t>
+          <t>0:46.8</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1662,7 @@
       <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>4:11</t>
+          <t>4:11.2</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>2:43.1</t>
+          <t>2:43.2</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>0:50.2</t>
+          <t>0:50.3</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>0:46.4</t>
+          <t>0:46.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a Halloween tag that shows as a pumpkin on a black chip
The tag is named Halloween in the song data (typeable for Muse and the
scripts) but displays as just 🎃: black filter chip (orange ring when
selected), black row pill, and a 🎃 chip in Add a song. Track list section
🎃 Halloween; AGENTS.md and submissions doc list it. Tests made label-aware
so tagging songs Halloween won't break them. No songs tagged yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2148,15 +2148,97 @@
       <c r="C94" s="2" t="inlineStr"/>
       <c r="D94" s="4" t="inlineStr"/>
     </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Army of Me</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3vEmpJQC2p8h0U3OiBufQm</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr"/>
+      <c r="D95" s="4" t="inlineStr"/>
+    </row>
     <row r="96">
-      <c r="A96" s="5" t="inlineStr">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Sphinx</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/6PhrbFbRW3Cchrv6klsLF5</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr"/>
+      <c r="D96" s="4" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>I Run</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/0DwJLxFUEBGr6jyIBaymlF</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr"/>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>0:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Livin' On A Prayer</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/37ZJ0p5Jm13JPevGcx4SkF</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr"/>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>1:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Zombie</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/49wOjOkS4pBK3PQnPnNYjb</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr"/>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>3:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss (or m:ss.s) and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D94"/>
+  <autoFilter ref="A1:D99"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2251,6 +2333,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" r:id="rId98"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Halloween start times on 10 songs; new Spooky Scary Skeletons link
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2230,15 +2230,271 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Beat It</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3BovdzfaX4jb5KFQwoPfAw</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>1:02</t>
+        </is>
+      </c>
+    </row>
     <row r="101">
-      <c r="A101" s="5" t="inlineStr">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Thriller</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/2LlQb7Uoj1kKyGhlkBf9aC</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>0:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Monster Mash</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/0xxZY5C9xxij3D1HkzbnfC</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>0:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Dracula</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/5adNBXEoLla10lGJcGzRIL</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>2:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Somebody's Watching Me</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/7jwQlYGpOml9ETGre1HqGA</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>1:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Spooky Scary Skeletons</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/2CfCbFpHnL3BYuV3VaY8Pl</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>0:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Hedwig's Theme</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/1n8NKQRg8LVHy7oUhUgbFF</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>1:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Ghostbusters</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/569uHYIB0X324FZOBEhvit</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>This Is Halloween</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3mhsDyQpX2L8sJMdWUHOi3</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>1:51.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>The Addams Family</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/00oHVAstyM08Q82e2XYvkS</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Halloween Theme</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/7swocJUCUWTCiRUAU9oerC</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>1:19.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Smooth Criminal</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/2bCQHF9gdG5BNDVuEIEnNk</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>1:31.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss (or m:ss.s) and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D99"/>
+  <autoFilter ref="A1:D111"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2338,6 +2594,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId110"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Halloween start-time tweaks, tag 2 songs Intermission, remove Celebration
Beat It 1:03; Dracula +0.4; Halloween Theme +0.2; Smooth Criminal +0.2;
Somebody's Watching Me +0.2; Spooky Scary Skeletons +0.1.
Intermission: 50 mission Cap, Believer. Removed: Celebration.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -489,7 +489,11 @@
           <t>https://open.spotify.com/track/0pqnGHJpmpxLKifKRmU6WP</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Intermission</t>
+        </is>
+      </c>
       <c r="D2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
@@ -1233,12 +1237,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Celebration</t>
+          <t>Hall of Fame</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3K7Q9PHUWPTaknlbFPThn2</t>
+          <t>https://open.spotify.com/track/7wMq5n8mYSKlQIGECKUgTX</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr"/>
@@ -1247,12 +1251,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Hall of Fame</t>
+          <t>Seven Nation Army</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7wMq5n8mYSKlQIGECKUgTX</t>
+          <t>https://open.spotify.com/track/3dPQuX8Gs42Y7b454ybpMR</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr"/>
@@ -1261,12 +1265,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Seven Nation Army</t>
+          <t>Freaks</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3dPQuX8Gs42Y7b454ybpMR</t>
+          <t>https://open.spotify.com/track/44DCjBHfvn5s6ZfLHpKmBi</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr"/>
@@ -1275,12 +1279,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Freaks</t>
+          <t>Play Hard</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/44DCjBHfvn5s6ZfLHpKmBi</t>
+          <t>https://open.spotify.com/track/5YPMEOJ58kfl56VHxTgwx3</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr"/>
@@ -1289,44 +1293,52 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Play Hard</t>
+          <t>The Gambler</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5YPMEOJ58kfl56VHxTgwx3</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/5KqldkCunQ2rWxruMEtGh0</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Penalty Kill</t>
+        </is>
+      </c>
       <c r="D48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>The Gambler</t>
+          <t>Born to be Wild</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5KqldkCunQ2rWxruMEtGh0</t>
+          <t>https://open.spotify.com/track/2VPGmrcBw5X4yAu3B8UZNE</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr"/>
+          <t>Wild</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>1:09.2</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Born to be Wild</t>
+          <t>Wild side</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2VPGmrcBw5X4yAu3B8UZNE</t>
+          <t>https://open.spotify.com/track/7zVpUAOuXY7pHHSm21jFEq</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -1336,19 +1348,19 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>1:09.2</t>
+          <t>2:46.1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Wild side</t>
+          <t>Wild one</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7zVpUAOuXY7pHHSm21jFEq</t>
+          <t>https://open.spotify.com/track/1NpW5kyvO4XrNJ3rnfcNy3</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -1358,73 +1370,73 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>2:46.1</t>
+          <t>2:02.5</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Wild one</t>
+          <t>Best day of my life</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1NpW5kyvO4XrNJ3rnfcNy3</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Wild</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>2:02.5</t>
+          <t>2:32.5</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Best day of my life</t>
+          <t>Sharp dressed man</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
+          <t>https://open.spotify.com/track/0bRNszTbTFLNlunAeh7eom</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr"/>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>2:32.5</t>
-        </is>
-      </c>
+      <c r="D53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Sharp dressed man</t>
+          <t>Hot to Go</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0bRNszTbTFLNlunAeh7eom</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="4" t="inlineStr"/>
+          <t>https://open.spotify.com/track/4xdBrk0nFZaP54vvZj0yx7</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>1:53.1</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Hot to Go</t>
+          <t>Giddy up</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4xdBrk0nFZaP54vvZj0yx7</t>
+          <t>https://open.spotify.com/track/4NdJlsPyvXz15LySCNoL2W</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -1434,185 +1446,185 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>1:53.1</t>
+          <t>0:32</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Giddy up</t>
+          <t>Man i feel like a woman</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4NdJlsPyvXz15LySCNoL2W</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Goal For</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>0:32</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/6sxptembJVty4sNtcPMAVz</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Man i feel like a woman</t>
+          <t>Venga Bus</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6sxptembJVty4sNtcPMAVz</t>
+          <t>https://open.spotify.com/track/73ljrkSg4A0q3ByU0Cu7mw</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr"/>
-      <c r="D57" s="4" t="inlineStr"/>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>1:09</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Venga Bus</t>
+          <t>Ceiling can't hold us</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/73ljrkSg4A0q3ByU0Cu7mw</t>
+          <t>https://open.spotify.com/track/22skzmqfdWrjJylampe0kt</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>1:09</t>
+          <t>3:49.5</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Ceiling can't hold us</t>
+          <t>Thunderstruck</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/22skzmqfdWrjJylampe0kt</t>
+          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>3:49.5</t>
+          <t>2:38.4</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Thunderstruck</t>
+          <t>Kickstart my Heart</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
+          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>2:38.4</t>
+          <t>1:03.3</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Kickstart my Heart</t>
+          <t>Shake it Off</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
+          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1:03.3</t>
+          <t>0:41.2</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Shake it Off</t>
+          <t>We're not gonna take it</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
+          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>0:41.2</t>
+          <t>0:46.8</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>We're not gonna take it</t>
+          <t>Fireball</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Power Play</t>
+        </is>
+      </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>0:46.8</t>
+          <t>1:32</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Fireball</t>
+          <t>I Did Something Bad</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Power Play</t>
+          <t>Penalty Kill</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>1:32</t>
+          <t>0:44</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>I Did Something Bad</t>
+          <t>Bad Girls</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
+          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -1622,257 +1634,257 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>0:44</t>
+          <t>1:36</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Bad Girls</t>
+          <t>Final Countdown</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Penalty Kill</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>1:36</t>
+          <t>4:11.2</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Final Countdown</t>
+          <t>Knights of Cydonia</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>4:11.2</t>
+          <t>4:13.2</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Knights of Cydonia</t>
+          <t>Immigrant Song</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
+          <t>https://open.spotify.com/track/78lgmZwycJ3nzsdgmPPGNx</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>4:13.2</t>
+          <t>0:01</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Immigrant Song</t>
+          <t>Fabienk</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/78lgmZwycJ3nzsdgmPPGNx</t>
+          <t>https://open.spotify.com/track/4UXwfhy8RTOcH0QWJF8SMg</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr"/>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>0:01</t>
+          <t>4:22</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Fabienk</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4UXwfhy8RTOcH0QWJF8SMg</t>
+          <t>https://open.spotify.com/track/1cp4LBTRjx98a6PjSCUFtL</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>4:22</t>
+          <t>2:10.2</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>Forget It</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1cp4LBTRjx98a6PjSCUFtL</t>
+          <t>https://open.spotify.com/track/7nbuGxQ7TfJXb9OgH3xJEr</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>2:10.2</t>
+          <t>0:40</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Forget It</t>
+          <t>Vogue</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7nbuGxQ7TfJXb9OgH3xJEr</t>
+          <t>https://open.spotify.com/track/1oE3n4VAn4of5vlVzJGynm</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr"/>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>0:40</t>
+          <t>2:43.2</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Vogue</t>
+          <t>September</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1oE3n4VAn4of5vlVzJGynm</t>
+          <t>https://open.spotify.com/track/748uyF14KEMCplV2CPAua7</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>2:43.2</t>
+          <t>0:50.3</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>Edge of Seventeen</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/748uyF14KEMCplV2CPAua7</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/7L3b6iaVhDVjfo52Hbvh9Z</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>End Game</t>
+        </is>
+      </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>0:50.3</t>
+          <t>4:17.5</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Edge of Seventeen</t>
+          <t>Billie Jean</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7L3b6iaVhDVjfo52Hbvh9Z</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>End Game</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/7J1uxwnxfQLu4APicE5Rnj</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr"/>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>4:17.5</t>
+          <t>1:26</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Billie Jean</t>
+          <t>Easy Lover</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7J1uxwnxfQLu4APicE5Rnj</t>
+          <t>https://open.spotify.com/track/5LYJ631w9ps5h9tdvac7yP</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr"/>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>1:26</t>
-        </is>
-      </c>
+      <c r="D76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Easy Lover</t>
+          <t>Black Betty</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5LYJ631w9ps5h9tdvac7yP</t>
+          <t>https://open.spotify.com/track/6kooDsorCpWVMGc994XjWN</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr"/>
-      <c r="D77" s="4" t="inlineStr"/>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>0:34</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Black Betty</t>
+          <t>Hero of the Day</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6kooDsorCpWVMGc994XjWN</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/2gF26K4auxwKMuWmLtO1io</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>End Game</t>
+        </is>
+      </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>0:34</t>
+          <t>0:37</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Hero of the Day</t>
+          <t>Hangar 18</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2gF26K4auxwKMuWmLtO1io</t>
+          <t>https://open.spotify.com/track/0KAaslGdPc5I6WxmKe3whe</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -1882,19 +1894,19 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>0:37</t>
+          <t>0:46.5</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Hangar 18</t>
+          <t>The Trooper</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0KAaslGdPc5I6WxmKe3whe</t>
+          <t>https://open.spotify.com/track/1W1Fchq0voTFhKGWmn57uW</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -1902,247 +1914,239 @@
           <t>End Game</t>
         </is>
       </c>
-      <c r="D80" s="4" t="inlineStr">
-        <is>
-          <t>0:46.5</t>
-        </is>
-      </c>
+      <c r="D80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>The Trooper</t>
+          <t>Stargazer</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1W1Fchq0voTFhKGWmn57uW</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>End Game</t>
-        </is>
-      </c>
-      <c r="D81" s="4" t="inlineStr"/>
+          <t>https://open.spotify.com/track/1aDNYyeU62BuQsBAY18i48</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr"/>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>0:08</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Stargazer</t>
+          <t>Seek &amp; Destroy</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1aDNYyeU62BuQsBAY18i48</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr"/>
-      <c r="D82" s="4" t="inlineStr">
-        <is>
-          <t>0:08</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/5DrNFzZZZVfXaEZCaceKnp</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Power Play, End Game</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Seek &amp; Destroy</t>
+          <t>Idioteque</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5DrNFzZZZVfXaEZCaceKnp</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>Power Play, End Game</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr"/>
+          <t>https://open.spotify.com/track/1W5XugQJGhnSATMI5n002M</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr"/>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>4:04</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Idioteque</t>
+          <t>Go With the Flow</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1W5XugQJGhnSATMI5n002M</t>
+          <t>https://open.spotify.com/track/45DElIx0dXqUH4A88yQFdE</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr"/>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>4:04</t>
-        </is>
-      </c>
+      <c r="D84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Go With the Flow</t>
+          <t>Lithium</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/45DElIx0dXqUH4A88yQFdE</t>
+          <t>https://open.spotify.com/track/2YodwKJnbPyNKe8XXSE9V7</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr"/>
-      <c r="D85" s="4" t="inlineStr"/>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>0:34</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Lithium</t>
+          <t>Mustache Man (Wasted)</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2YodwKJnbPyNKe8XXSE9V7</t>
+          <t>https://open.spotify.com/track/5YfE7GXM5Mfs9Aul3uth1j</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr"/>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>0:34</t>
-        </is>
-      </c>
+      <c r="D86" s="4" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Mustache Man (Wasted)</t>
+          <t>Turn The Lights Off</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5YfE7GXM5Mfs9Aul3uth1j</t>
+          <t>https://open.spotify.com/track/0wHayguZd1CeQDLYohXNMS</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr"/>
-      <c r="D87" s="4" t="inlineStr"/>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>2:25</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Turn The Lights Off</t>
+          <t>Misty Mountain Hop</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0wHayguZd1CeQDLYohXNMS</t>
+          <t>https://open.spotify.com/track/3frf3zTgzt3YIx9ylpUoqU</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr"/>
-      <c r="D88" s="4" t="inlineStr">
-        <is>
-          <t>2:25</t>
-        </is>
-      </c>
+      <c r="D88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Misty Mountain Hop</t>
+          <t>No Broke Boys</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3frf3zTgzt3YIx9ylpUoqU</t>
+          <t>https://open.spotify.com/track/3cZajhyr8LmtPfHZ9296tj</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr"/>
-      <c r="D89" s="4" t="inlineStr"/>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>0:30</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>No Broke Boys</t>
+          <t>Goal horn</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3cZajhyr8LmtPfHZ9296tj</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr"/>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/7gfcVjQLq4lKObJD6dU7r7</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Goal horn</t>
+          <t>crowd chant</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7gfcVjQLq4lKObJD6dU7r7</t>
+          <t>https://open.spotify.com/track/0bz67HYKfiuUj1xhsK5ofT</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Goal For</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr"/>
+          <t>Power Play, Goal For</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>0:24</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>crowd chant</t>
+          <t>50 mission Cap</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0bz67HYKfiuUj1xhsK5ofT</t>
+          <t>https://open.spotify.com/track/6UA5wCnNHbPZzT1O0tWQy0</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Power Play, Goal For</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>0:24</t>
-        </is>
-      </c>
+          <t>Power Play, Intermission</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>50 mission Cap</t>
+          <t>you've got another thing coming</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6UA5wCnNHbPZzT1O0tWQy0</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>Power Play</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/4f3RDq9nYPBeR1yMSgnmBm</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr"/>
       <c r="D93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>you've got another thing coming</t>
+          <t>Army of Me</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4f3RDq9nYPBeR1yMSgnmBm</t>
+          <t>https://open.spotify.com/track/3vEmpJQC2p8h0U3OiBufQm</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr"/>
@@ -2151,12 +2155,12 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Army of Me</t>
+          <t>Sphinx</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3vEmpJQC2p8h0U3OiBufQm</t>
+          <t>https://open.spotify.com/track/6PhrbFbRW3Cchrv6klsLF5</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr"/>
@@ -2165,80 +2169,88 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Sphinx</t>
+          <t>I Run</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6PhrbFbRW3Cchrv6klsLF5</t>
+          <t>https://open.spotify.com/track/0DwJLxFUEBGr6jyIBaymlF</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr"/>
-      <c r="D96" s="4" t="inlineStr"/>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>0:28</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>I Run</t>
+          <t>Livin' On A Prayer</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0DwJLxFUEBGr6jyIBaymlF</t>
+          <t>https://open.spotify.com/track/37ZJ0p5Jm13JPevGcx4SkF</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr"/>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>0:28</t>
+          <t>1:33</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Livin' On A Prayer</t>
+          <t>Zombie</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/37ZJ0p5Jm13JPevGcx4SkF</t>
+          <t>https://open.spotify.com/track/49wOjOkS4pBK3PQnPnNYjb</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr"/>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>1:33</t>
+          <t>3:06</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Zombie</t>
+          <t>Beat It</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/49wOjOkS4pBK3PQnPnNYjb</t>
-        </is>
-      </c>
-      <c r="C99" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/3BovdzfaX4jb5KFQwoPfAw</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>3:06</t>
+          <t>1:03</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Beat It</t>
+          <t>Thriller</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3BovdzfaX4jb5KFQwoPfAw</t>
+          <t>https://open.spotify.com/track/2LlQb7Uoj1kKyGhlkBf9aC</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -2248,19 +2260,19 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>1:02</t>
+          <t>0:36</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Thriller</t>
+          <t>Monster Mash</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2LlQb7Uoj1kKyGhlkBf9aC</t>
+          <t>https://open.spotify.com/track/0xxZY5C9xxij3D1HkzbnfC</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -2270,19 +2282,19 @@
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>0:36</t>
+          <t>0:56</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Monster Mash</t>
+          <t>Dracula</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0xxZY5C9xxij3D1HkzbnfC</t>
+          <t>https://open.spotify.com/track/5adNBXEoLla10lGJcGzRIL</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -2292,19 +2304,19 @@
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>0:56</t>
+          <t>2:40.4</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Dracula</t>
+          <t>Somebody's Watching Me</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5adNBXEoLla10lGJcGzRIL</t>
+          <t>https://open.spotify.com/track/7jwQlYGpOml9ETGre1HqGA</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -2314,19 +2326,19 @@
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>2:40</t>
+          <t>1:36.2</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Somebody's Watching Me</t>
+          <t>Spooky Scary Skeletons</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7jwQlYGpOml9ETGre1HqGA</t>
+          <t>https://open.spotify.com/track/2CfCbFpHnL3BYuV3VaY8Pl</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -2336,19 +2348,19 @@
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>1:36</t>
+          <t>0:07.1</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Spooky Scary Skeletons</t>
+          <t>Hedwig's Theme</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2CfCbFpHnL3BYuV3VaY8Pl</t>
+          <t>https://open.spotify.com/track/1n8NKQRg8LVHy7oUhUgbFF</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -2358,19 +2370,19 @@
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>0:07</t>
+          <t>1:18</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Hedwig's Theme</t>
+          <t>Ghostbusters</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1n8NKQRg8LVHy7oUhUgbFF</t>
+          <t>https://open.spotify.com/track/569uHYIB0X324FZOBEhvit</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -2378,21 +2390,17 @@
           <t>Halloween</t>
         </is>
       </c>
-      <c r="D106" s="4" t="inlineStr">
-        <is>
-          <t>1:18</t>
-        </is>
-      </c>
+      <c r="D106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Ghostbusters</t>
+          <t>This Is Halloween</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/569uHYIB0X324FZOBEhvit</t>
+          <t>https://open.spotify.com/track/3mhsDyQpX2L8sJMdWUHOi3</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -2400,17 +2408,21 @@
           <t>Halloween</t>
         </is>
       </c>
-      <c r="D107" s="4" t="inlineStr"/>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>1:51.2</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>This Is Halloween</t>
+          <t>The Addams Family</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3mhsDyQpX2L8sJMdWUHOi3</t>
+          <t>https://open.spotify.com/track/00oHVAstyM08Q82e2XYvkS</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -2418,21 +2430,17 @@
           <t>Halloween</t>
         </is>
       </c>
-      <c r="D108" s="4" t="inlineStr">
-        <is>
-          <t>1:51.2</t>
-        </is>
-      </c>
+      <c r="D108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>The Addams Family</t>
+          <t>Halloween Theme</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/00oHVAstyM08Q82e2XYvkS</t>
+          <t>https://open.spotify.com/track/7swocJUCUWTCiRUAU9oerC</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -2440,17 +2448,21 @@
           <t>Halloween</t>
         </is>
       </c>
-      <c r="D109" s="4" t="inlineStr"/>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>1:20.1</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Halloween Theme</t>
+          <t>Smooth Criminal</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7swocJUCUWTCiRUAU9oerC</t>
+          <t>https://open.spotify.com/track/2bCQHF9gdG5BNDVuEIEnNk</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -2460,41 +2472,19 @@
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>1:19.9</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>Smooth Criminal</t>
-        </is>
-      </c>
-      <c r="B111" s="3" t="inlineStr">
-        <is>
-          <t>https://open.spotify.com/track/2bCQHF9gdG5BNDVuEIEnNk</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>Halloween</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>1:31.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="5" t="inlineStr">
+          <t>1:31.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss (or m:ss.s) and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D111"/>
+  <autoFilter ref="A1:D110"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2605,7 +2595,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B108" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId110"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Intermission x5, Goal For: Kernkraft 400, End Game: Narco; add Go Go Girl and Girls Rule; Seven Nation Army 0:47
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D112"/>
+  <dimension ref="A1:D114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -525,7 +525,11 @@
           <t>https://open.spotify.com/track/6RSuGXM9GVMdXaI8ifGm8d</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Intermission</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -577,7 +581,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>End Game</t>
+          <t>End Game, Intermission</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -651,7 +655,11 @@
           <t>https://open.spotify.com/track/1vLqigPHwiFnXsfrLMehV1</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Intermission</t>
+        </is>
+      </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
           <t>0:08</t>
@@ -969,7 +977,11 @@
           <t>https://open.spotify.com/track/3SWqGa1J0M7hSBUDM0KePD</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Intermission</t>
+        </is>
+      </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
           <t>0:16</t>
@@ -1001,7 +1013,11 @@
           <t>https://open.spotify.com/track/3f2fyR55BFMl3ZWS5S3BUZ</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
           <t>1:56</t>
@@ -1161,7 +1177,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
+          <t>Penalty Kill, End Game</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr"/>
@@ -1245,7 +1261,11 @@
           <t>https://open.spotify.com/track/7wMq5n8mYSKlQIGECKUgTX</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Intermission</t>
+        </is>
+      </c>
       <c r="D44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
@@ -1260,7 +1280,11 @@
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>0:47</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2476,15 +2500,55 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Go Go Girl</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/0OhRzvfoqTLkWGE0J2mWh2</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>2:04.9</t>
+        </is>
+      </c>
+    </row>
     <row r="112">
-      <c r="A112" s="5" t="inlineStr">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Girls Rule</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3IITulnaPefCg6buu079oy</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr"/>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>0:50.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss (or m:ss.s) and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D110"/>
+  <autoFilter ref="A1:D112"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2595,6 +2659,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B108" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B112" r:id="rId111"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Bring Em Out, Tsunami, Titanium, Deuces are Wild (Wild); remove The Gambler; We're not gonna take it -> Goal Against; Thunder +0.3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$115</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D114"/>
+  <dimension ref="A1:D117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1196,7 +1196,7 @@
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>1:13.8</t>
+          <t>1:14.1</t>
         </is>
       </c>
     </row>
@@ -1317,30 +1317,34 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>The Gambler</t>
+          <t>Born to be Wild</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5KqldkCunQ2rWxruMEtGh0</t>
+          <t>https://open.spotify.com/track/2VPGmrcBw5X4yAu3B8UZNE</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr"/>
+          <t>Wild</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>1:09.2</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Born to be Wild</t>
+          <t>Wild side</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2VPGmrcBw5X4yAu3B8UZNE</t>
+          <t>https://open.spotify.com/track/7zVpUAOuXY7pHHSm21jFEq</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -1350,19 +1354,19 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>1:09.2</t>
+          <t>2:46.1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Wild side</t>
+          <t>Wild one</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7zVpUAOuXY7pHHSm21jFEq</t>
+          <t>https://open.spotify.com/track/1NpW5kyvO4XrNJ3rnfcNy3</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -1372,73 +1376,73 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>2:46.1</t>
+          <t>2:02.5</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Wild one</t>
+          <t>Best day of my life</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1NpW5kyvO4XrNJ3rnfcNy3</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Wild</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>2:02.5</t>
+          <t>2:32.5</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Best day of my life</t>
+          <t>Sharp dressed man</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5Hroj5K7vLpIG4FNCRIjbP</t>
+          <t>https://open.spotify.com/track/0bRNszTbTFLNlunAeh7eom</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>2:32.5</t>
-        </is>
-      </c>
+      <c r="D52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Sharp dressed man</t>
+          <t>Hot to Go</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0bRNszTbTFLNlunAeh7eom</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr"/>
-      <c r="D53" s="4" t="inlineStr"/>
+          <t>https://open.spotify.com/track/4xdBrk0nFZaP54vvZj0yx7</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>1:53.1</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Hot to Go</t>
+          <t>Giddy up</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4xdBrk0nFZaP54vvZj0yx7</t>
+          <t>https://open.spotify.com/track/4NdJlsPyvXz15LySCNoL2W</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -1448,185 +1452,189 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>1:53.1</t>
+          <t>0:32</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Giddy up</t>
+          <t>Man i feel like a woman</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4NdJlsPyvXz15LySCNoL2W</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Goal For</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>0:32</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/6sxptembJVty4sNtcPMAVz</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Man i feel like a woman</t>
+          <t>Venga Bus</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6sxptembJVty4sNtcPMAVz</t>
+          <t>https://open.spotify.com/track/73ljrkSg4A0q3ByU0Cu7mw</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="4" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>1:09</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Venga Bus</t>
+          <t>Ceiling can't hold us</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/73ljrkSg4A0q3ByU0Cu7mw</t>
+          <t>https://open.spotify.com/track/22skzmqfdWrjJylampe0kt</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr"/>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>1:09</t>
+          <t>3:49.5</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Ceiling can't hold us</t>
+          <t>Thunderstruck</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/22skzmqfdWrjJylampe0kt</t>
+          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>3:49.5</t>
+          <t>2:38.4</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Thunderstruck</t>
+          <t>Kickstart my Heart</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
+          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>2:38.4</t>
+          <t>1:03.3</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Kickstart my Heart</t>
+          <t>Shake it Off</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
+          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>1:03.3</t>
+          <t>0:41.2</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Shake it Off</t>
+          <t>We're not gonna take it</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Goal Against</t>
+        </is>
+      </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>0:41.2</t>
+          <t>0:46.8</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>We're not gonna take it</t>
+          <t>Fireball</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Power Play</t>
+        </is>
+      </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>0:46.8</t>
+          <t>1:32</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Fireball</t>
+          <t>I Did Something Bad</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Power Play</t>
+          <t>Penalty Kill</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>1:32</t>
+          <t>0:44</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>I Did Something Bad</t>
+          <t>Bad Girls</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
+          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -1636,257 +1644,257 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>0:44</t>
+          <t>1:36</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Bad Girls</t>
+          <t>Final Countdown</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Penalty Kill</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>1:36</t>
+          <t>4:11.2</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Final Countdown</t>
+          <t>Knights of Cydonia</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>4:11.2</t>
+          <t>4:13.2</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Knights of Cydonia</t>
+          <t>Immigrant Song</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
+          <t>https://open.spotify.com/track/78lgmZwycJ3nzsdgmPPGNx</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>4:13.2</t>
+          <t>0:01</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Immigrant Song</t>
+          <t>Fabienk</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/78lgmZwycJ3nzsdgmPPGNx</t>
+          <t>https://open.spotify.com/track/4UXwfhy8RTOcH0QWJF8SMg</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>0:01</t>
+          <t>4:22</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Fabienk</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4UXwfhy8RTOcH0QWJF8SMg</t>
+          <t>https://open.spotify.com/track/1cp4LBTRjx98a6PjSCUFtL</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr"/>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>4:22</t>
+          <t>2:10.2</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>Forget It</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1cp4LBTRjx98a6PjSCUFtL</t>
+          <t>https://open.spotify.com/track/7nbuGxQ7TfJXb9OgH3xJEr</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>2:10.2</t>
+          <t>0:40</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Forget It</t>
+          <t>Vogue</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7nbuGxQ7TfJXb9OgH3xJEr</t>
+          <t>https://open.spotify.com/track/1oE3n4VAn4of5vlVzJGynm</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>0:40</t>
+          <t>2:43.2</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Vogue</t>
+          <t>September</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1oE3n4VAn4of5vlVzJGynm</t>
+          <t>https://open.spotify.com/track/748uyF14KEMCplV2CPAua7</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr"/>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>2:43.2</t>
+          <t>0:50.3</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>Edge of Seventeen</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/748uyF14KEMCplV2CPAua7</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/7L3b6iaVhDVjfo52Hbvh9Z</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>End Game</t>
+        </is>
+      </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>0:50.3</t>
+          <t>4:17.5</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Edge of Seventeen</t>
+          <t>Billie Jean</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7L3b6iaVhDVjfo52Hbvh9Z</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>End Game</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/7J1uxwnxfQLu4APicE5Rnj</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>4:17.5</t>
+          <t>1:26</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Billie Jean</t>
+          <t>Easy Lover</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7J1uxwnxfQLu4APicE5Rnj</t>
+          <t>https://open.spotify.com/track/5LYJ631w9ps5h9tdvac7yP</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr"/>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>1:26</t>
-        </is>
-      </c>
+      <c r="D75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Easy Lover</t>
+          <t>Black Betty</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5LYJ631w9ps5h9tdvac7yP</t>
+          <t>https://open.spotify.com/track/6kooDsorCpWVMGc994XjWN</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr"/>
-      <c r="D76" s="4" t="inlineStr"/>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>0:34</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Black Betty</t>
+          <t>Hero of the Day</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6kooDsorCpWVMGc994XjWN</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/2gF26K4auxwKMuWmLtO1io</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>End Game</t>
+        </is>
+      </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>0:34</t>
+          <t>0:37</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Hero of the Day</t>
+          <t>Hangar 18</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2gF26K4auxwKMuWmLtO1io</t>
+          <t>https://open.spotify.com/track/0KAaslGdPc5I6WxmKe3whe</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -1896,19 +1904,19 @@
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>0:37</t>
+          <t>0:46.5</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Hangar 18</t>
+          <t>The Trooper</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0KAaslGdPc5I6WxmKe3whe</t>
+          <t>https://open.spotify.com/track/1W1Fchq0voTFhKGWmn57uW</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -1916,247 +1924,239 @@
           <t>End Game</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>0:46.5</t>
-        </is>
-      </c>
+      <c r="D79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>The Trooper</t>
+          <t>Stargazer</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1W1Fchq0voTFhKGWmn57uW</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>End Game</t>
-        </is>
-      </c>
-      <c r="D80" s="4" t="inlineStr"/>
+          <t>https://open.spotify.com/track/1aDNYyeU62BuQsBAY18i48</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr"/>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>0:08</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Stargazer</t>
+          <t>Seek &amp; Destroy</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1aDNYyeU62BuQsBAY18i48</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr"/>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>0:08</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/5DrNFzZZZVfXaEZCaceKnp</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Power Play, End Game</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Seek &amp; Destroy</t>
+          <t>Idioteque</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5DrNFzZZZVfXaEZCaceKnp</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>Power Play, End Game</t>
-        </is>
-      </c>
-      <c r="D82" s="4" t="inlineStr"/>
+          <t>https://open.spotify.com/track/1W5XugQJGhnSATMI5n002M</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr"/>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>4:04</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Idioteque</t>
+          <t>Go With the Flow</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1W5XugQJGhnSATMI5n002M</t>
+          <t>https://open.spotify.com/track/45DElIx0dXqUH4A88yQFdE</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr"/>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>4:04</t>
-        </is>
-      </c>
+      <c r="D83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Go With the Flow</t>
+          <t>Lithium</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/45DElIx0dXqUH4A88yQFdE</t>
+          <t>https://open.spotify.com/track/2YodwKJnbPyNKe8XXSE9V7</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr"/>
-      <c r="D84" s="4" t="inlineStr"/>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>0:34</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Lithium</t>
+          <t>Mustache Man (Wasted)</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2YodwKJnbPyNKe8XXSE9V7</t>
+          <t>https://open.spotify.com/track/5YfE7GXM5Mfs9Aul3uth1j</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr"/>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>0:34</t>
-        </is>
-      </c>
+      <c r="D85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Mustache Man (Wasted)</t>
+          <t>Turn The Lights Off</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5YfE7GXM5Mfs9Aul3uth1j</t>
+          <t>https://open.spotify.com/track/0wHayguZd1CeQDLYohXNMS</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr"/>
-      <c r="D86" s="4" t="inlineStr"/>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>2:25</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Turn The Lights Off</t>
+          <t>Misty Mountain Hop</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0wHayguZd1CeQDLYohXNMS</t>
+          <t>https://open.spotify.com/track/3frf3zTgzt3YIx9ylpUoqU</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr"/>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>2:25</t>
-        </is>
-      </c>
+      <c r="D87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Misty Mountain Hop</t>
+          <t>No Broke Boys</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3frf3zTgzt3YIx9ylpUoqU</t>
+          <t>https://open.spotify.com/track/3cZajhyr8LmtPfHZ9296tj</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr"/>
-      <c r="D88" s="4" t="inlineStr"/>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>0:30</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>No Broke Boys</t>
+          <t>Goal horn</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3cZajhyr8LmtPfHZ9296tj</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr"/>
-      <c r="D89" s="4" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/7gfcVjQLq4lKObJD6dU7r7</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Goal horn</t>
+          <t>crowd chant</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7gfcVjQLq4lKObJD6dU7r7</t>
+          <t>https://open.spotify.com/track/0bz67HYKfiuUj1xhsK5ofT</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Goal For</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr"/>
+          <t>Power Play, Goal For</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>0:24</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>crowd chant</t>
+          <t>50 mission Cap</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0bz67HYKfiuUj1xhsK5ofT</t>
+          <t>https://open.spotify.com/track/6UA5wCnNHbPZzT1O0tWQy0</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Power Play, Goal For</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>0:24</t>
-        </is>
-      </c>
+          <t>Power Play, Intermission</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>50 mission Cap</t>
+          <t>you've got another thing coming</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6UA5wCnNHbPZzT1O0tWQy0</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>Power Play, Intermission</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/4f3RDq9nYPBeR1yMSgnmBm</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr"/>
       <c r="D92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>you've got another thing coming</t>
+          <t>Army of Me</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4f3RDq9nYPBeR1yMSgnmBm</t>
+          <t>https://open.spotify.com/track/3vEmpJQC2p8h0U3OiBufQm</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr"/>
@@ -2165,12 +2165,12 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Army of Me</t>
+          <t>Sphinx</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3vEmpJQC2p8h0U3OiBufQm</t>
+          <t>https://open.spotify.com/track/6PhrbFbRW3Cchrv6klsLF5</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr"/>
@@ -2179,80 +2179,88 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Sphinx</t>
+          <t>I Run</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/6PhrbFbRW3Cchrv6klsLF5</t>
+          <t>https://open.spotify.com/track/0DwJLxFUEBGr6jyIBaymlF</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr"/>
-      <c r="D95" s="4" t="inlineStr"/>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>0:28</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>I Run</t>
+          <t>Livin' On A Prayer</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0DwJLxFUEBGr6jyIBaymlF</t>
+          <t>https://open.spotify.com/track/37ZJ0p5Jm13JPevGcx4SkF</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr"/>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>0:28</t>
+          <t>1:33</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Livin' On A Prayer</t>
+          <t>Zombie</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/37ZJ0p5Jm13JPevGcx4SkF</t>
+          <t>https://open.spotify.com/track/49wOjOkS4pBK3PQnPnNYjb</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr"/>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>1:33</t>
+          <t>3:06</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Zombie</t>
+          <t>Beat It</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/49wOjOkS4pBK3PQnPnNYjb</t>
-        </is>
-      </c>
-      <c r="C98" s="2" t="inlineStr"/>
+          <t>https://open.spotify.com/track/3BovdzfaX4jb5KFQwoPfAw</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Halloween</t>
+        </is>
+      </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>3:06</t>
+          <t>1:03</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Beat It</t>
+          <t>Thriller</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3BovdzfaX4jb5KFQwoPfAw</t>
+          <t>https://open.spotify.com/track/2LlQb7Uoj1kKyGhlkBf9aC</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -2262,19 +2270,19 @@
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>1:03</t>
+          <t>0:36</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Thriller</t>
+          <t>Monster Mash</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2LlQb7Uoj1kKyGhlkBf9aC</t>
+          <t>https://open.spotify.com/track/0xxZY5C9xxij3D1HkzbnfC</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -2284,19 +2292,19 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>0:36</t>
+          <t>0:56</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Monster Mash</t>
+          <t>Dracula</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0xxZY5C9xxij3D1HkzbnfC</t>
+          <t>https://open.spotify.com/track/5adNBXEoLla10lGJcGzRIL</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -2306,19 +2314,19 @@
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>0:56</t>
+          <t>2:40.4</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Dracula</t>
+          <t>Somebody's Watching Me</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5adNBXEoLla10lGJcGzRIL</t>
+          <t>https://open.spotify.com/track/7jwQlYGpOml9ETGre1HqGA</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -2328,19 +2336,19 @@
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>2:40.4</t>
+          <t>1:36.2</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Somebody's Watching Me</t>
+          <t>Spooky Scary Skeletons</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7jwQlYGpOml9ETGre1HqGA</t>
+          <t>https://open.spotify.com/track/2CfCbFpHnL3BYuV3VaY8Pl</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -2350,19 +2358,19 @@
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>1:36.2</t>
+          <t>0:07.1</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Spooky Scary Skeletons</t>
+          <t>Hedwig's Theme</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2CfCbFpHnL3BYuV3VaY8Pl</t>
+          <t>https://open.spotify.com/track/1n8NKQRg8LVHy7oUhUgbFF</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -2372,19 +2380,19 @@
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>0:07.1</t>
+          <t>1:18</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Hedwig's Theme</t>
+          <t>Ghostbusters</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1n8NKQRg8LVHy7oUhUgbFF</t>
+          <t>https://open.spotify.com/track/569uHYIB0X324FZOBEhvit</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -2392,21 +2400,17 @@
           <t>Halloween</t>
         </is>
       </c>
-      <c r="D105" s="4" t="inlineStr">
-        <is>
-          <t>1:18</t>
-        </is>
-      </c>
+      <c r="D105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Ghostbusters</t>
+          <t>This Is Halloween</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/569uHYIB0X324FZOBEhvit</t>
+          <t>https://open.spotify.com/track/3mhsDyQpX2L8sJMdWUHOi3</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -2414,17 +2418,21 @@
           <t>Halloween</t>
         </is>
       </c>
-      <c r="D106" s="4" t="inlineStr"/>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>1:51.2</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>This Is Halloween</t>
+          <t>The Addams Family</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3mhsDyQpX2L8sJMdWUHOi3</t>
+          <t>https://open.spotify.com/track/00oHVAstyM08Q82e2XYvkS</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -2432,21 +2440,17 @@
           <t>Halloween</t>
         </is>
       </c>
-      <c r="D107" s="4" t="inlineStr">
-        <is>
-          <t>1:51.2</t>
-        </is>
-      </c>
+      <c r="D107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>The Addams Family</t>
+          <t>Halloween Theme</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/00oHVAstyM08Q82e2XYvkS</t>
+          <t>https://open.spotify.com/track/7swocJUCUWTCiRUAU9oerC</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -2454,17 +2458,21 @@
           <t>Halloween</t>
         </is>
       </c>
-      <c r="D108" s="4" t="inlineStr"/>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>1:20.1</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Halloween Theme</t>
+          <t>Smooth Criminal</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7swocJUCUWTCiRUAU9oerC</t>
+          <t>https://open.spotify.com/track/2bCQHF9gdG5BNDVuEIEnNk</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -2474,81 +2482,135 @@
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>1:20.1</t>
+          <t>1:31.7</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Smooth Criminal</t>
+          <t>Go Go Girl</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/2bCQHF9gdG5BNDVuEIEnNk</t>
+          <t>https://open.spotify.com/track/0OhRzvfoqTLkWGE0J2mWh2</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Halloween</t>
+          <t>Goal For</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>1:31.7</t>
+          <t>2:04.9</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Go Go Girl</t>
+          <t>Girls Rule</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/0OhRzvfoqTLkWGE0J2mWh2</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>Goal For</t>
-        </is>
-      </c>
+          <t>https://open.spotify.com/track/3IITulnaPefCg6buu079oy</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr"/>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>2:04.9</t>
+          <t>0:50.2</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Girls Rule</t>
+          <t>Bring Em Out</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3IITulnaPefCg6buu079oy</t>
+          <t>https://open.spotify.com/track/7oAZVxmRCVFanxK7tk16vv</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr"/>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>0:50.2</t>
+          <t>1:23.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Tsunami</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/0u4SRuld2zPAnyImNdfMAo</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr"/>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>1:14.7</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="5" t="inlineStr">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Titanium</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/0lHAMNU8RGiIObScrsRgmP</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr"/>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>1:09.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Deuces are Wild</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/1Xc6m2d5iReJCuWTJLBtBG</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Wild</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>2:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.SONGS block in index.html. Tags are blank for a between-whistles song. Start Time is shown as m:ss (or m:ss.s) and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D112"/>
+  <autoFilter ref="A1:D115"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2661,6 +2723,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId109"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId114"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Turn The Lights Off -> Goal Against
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -2037,7 +2037,11 @@
           <t>https://open.spotify.com/track/0wHayguZd1CeQDLYohXNMS</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr"/>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Goal Against</t>
+        </is>
+      </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
           <t>2:25</t>

</xml_diff>

<commit_message>
This Is Halloween +0.2, Monster Mash +0.2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -2296,7 +2296,7 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>0:56</t>
+          <t>0:56.2</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>1:51.2</t>
+          <t>1:51.4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Zombie -> Zombie WRENN, tagged Goal For
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -2219,7 +2219,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Zombie</t>
+          <t>Zombie WRENN</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -2227,7 +2227,11 @@
           <t>https://open.spotify.com/track/49wOjOkS4pBK3PQnPnNYjb</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr"/>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Goal For</t>
+        </is>
+      </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
           <t>3:06</t>

</xml_diff>

<commit_message>
New Banger tag (electric cyan, BNG) on 7 songs; Goal Against +2; title-case all song names
Banger: Go with the Flow, Brutal, Easy Lover, Lithium, Sharp Dressed Man,
Stargazer, You've Got Another Thing Coming.
Goal Against: + Shake It Off, Forget It (We're Not Gonna Take It already had it).
31 song names title-cased (small words like a/the/of/on/with stay lowercase
mid-title; all-caps names like YYZ and WRENN kept).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013MToeLQag51itynxiSUTyb
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -687,7 +687,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>brutal</t>
+          <t>Brutal</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -695,7 +695,11 @@
           <t>https://open.spotify.com/track/6SRsiMl7w1USE4mFqrOhHC</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Banger</t>
+        </is>
+      </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
           <t>1:00.5</t>
@@ -723,7 +727,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Wild child</t>
+          <t>Wild Child</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -763,7 +767,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Chelsea dagger</t>
+          <t>Chelsea Dagger</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -843,7 +847,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>pink pony club</t>
+          <t>Pink Pony Club</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -861,7 +865,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>the distance</t>
+          <t>The Distance</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -879,7 +883,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>wild thing</t>
+          <t>Wild Thing</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -897,7 +901,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>brass</t>
+          <t>Brass</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -915,7 +919,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>get ready for this</t>
+          <t>Get Ready for This</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -933,7 +937,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>handclap</t>
+          <t>Handclap</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -951,7 +955,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>rock n roll gary glitter</t>
+          <t>Rock N Roll Gary Glitter</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -969,7 +973,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>legend</t>
+          <t>Legend</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1203,7 +1207,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Miles On It</t>
+          <t>Miles on It</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1317,7 +1321,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Born to be Wild</t>
+          <t>Born to Be Wild</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1339,7 +1343,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Wild side</t>
+          <t>Wild Side</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1361,7 +1365,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Wild one</t>
+          <t>Wild One</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1383,7 +1387,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Best day of my life</t>
+          <t>Best Day of My Life</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1401,7 +1405,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Sharp dressed man</t>
+          <t>Sharp Dressed Man</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -1409,7 +1413,11 @@
           <t>https://open.spotify.com/track/0bRNszTbTFLNlunAeh7eom</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Banger</t>
+        </is>
+      </c>
       <c r="D52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
@@ -1437,7 +1445,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Giddy up</t>
+          <t>Giddy Up</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1459,7 +1467,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Man i feel like a woman</t>
+          <t>Man I Feel Like a Woman</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1491,7 +1499,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Ceiling can't hold us</t>
+          <t>Ceiling Can't Hold Us</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -1527,7 +1535,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Kickstart my Heart</t>
+          <t>Kickstart My Heart</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -1545,7 +1553,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Shake it Off</t>
+          <t>Shake It Off</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -1553,7 +1561,11 @@
           <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr"/>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Goal Against</t>
+        </is>
+      </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
           <t>0:41.2</t>
@@ -1563,7 +1575,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>We're not gonna take it</t>
+          <t>We're Not Gonna Take It</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -1749,7 +1761,11 @@
           <t>https://open.spotify.com/track/7nbuGxQ7TfJXb9OgH3xJEr</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr"/>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Goal Against</t>
+        </is>
+      </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
           <t>0:40</t>
@@ -1843,7 +1859,11 @@
           <t>https://open.spotify.com/track/5LYJ631w9ps5h9tdvac7yP</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr"/>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Banger</t>
+        </is>
+      </c>
       <c r="D75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
@@ -1937,7 +1957,11 @@
           <t>https://open.spotify.com/track/1aDNYyeU62BuQsBAY18i48</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr"/>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Banger</t>
+        </is>
+      </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
           <t>0:08</t>
@@ -1983,7 +2007,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Go With the Flow</t>
+          <t>Go with the Flow</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -1991,7 +2015,11 @@
           <t>https://open.spotify.com/track/45DElIx0dXqUH4A88yQFdE</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr"/>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Banger</t>
+        </is>
+      </c>
       <c r="D83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
@@ -2005,7 +2033,11 @@
           <t>https://open.spotify.com/track/2YodwKJnbPyNKe8XXSE9V7</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr"/>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Banger</t>
+        </is>
+      </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
           <t>0:34</t>
@@ -2029,7 +2061,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Turn The Lights Off</t>
+          <t>Turn the Lights Off</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -2083,7 +2115,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Goal horn</t>
+          <t>Goal Horn</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -2101,7 +2133,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>crowd chant</t>
+          <t>Crowd Chant</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -2123,7 +2155,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>50 mission Cap</t>
+          <t>50 Mission Cap</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -2141,7 +2173,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>you've got another thing coming</t>
+          <t>You've Got Another Thing Coming</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -2149,7 +2181,11 @@
           <t>https://open.spotify.com/track/4f3RDq9nYPBeR1yMSgnmBm</t>
         </is>
       </c>
-      <c r="C92" s="2" t="inlineStr"/>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Banger</t>
+        </is>
+      </c>
       <c r="D92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
@@ -2201,7 +2237,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Livin' On A Prayer</t>
+          <t>Livin' on a Prayer</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -2591,7 +2627,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Deuces are Wild</t>
+          <t>Deuces Are Wild</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">

</xml_diff>